<commit_message>
Added - Cardboard plant art
</commit_message>
<xml_diff>
--- a/art/art_direction.xlsx
+++ b/art/art_direction.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\art\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397FE321-F5D9-4897-8E87-FECF93922A1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7855133D-65E5-4088-B0AF-EC9DFC0BD303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4770" yWindow="-21600" windowWidth="36555" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20040" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General Usages" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="82">
   <si>
     <t>Black</t>
   </si>
@@ -266,6 +266,12 @@
   </si>
   <si>
     <t>Poison</t>
+  </si>
+  <si>
+    <t>Cardboard</t>
+  </si>
+  <si>
+    <t>04</t>
   </si>
 </sst>
 </file>
@@ -631,7 +637,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.21875" style="3" customWidth="1"/>
@@ -700,182 +706,190 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>13</v>
+        <v>80</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M6" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M7" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M9" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+    <row r="10" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M10" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L10" s="4" t="s">
+      <c r="L11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M11" s="4" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="M13" s="4" t="s">
+      <c r="C14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M14" s="4" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="M16" s="4" t="s">
-        <v>45</v>
+        <v>79</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M18" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
+    <row r="19" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="E19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="M20" s="4" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G20" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L20" s="4" t="s">
+      <c r="G21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="L21" s="4" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M20">
-    <sortCondition ref="A1:A20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M21">
+    <sortCondition ref="A1:A21"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Added - Grow-shroom art
</commit_message>
<xml_diff>
--- a/art/art_direction.xlsx
+++ b/art/art_direction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\art\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7855133D-65E5-4088-B0AF-EC9DFC0BD303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85AEE0C4-3B63-422A-8F25-93E9982FE4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20040" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General Usages" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="84">
   <si>
     <t>Black</t>
   </si>
@@ -272,6 +272,12 @@
   </si>
   <si>
     <t>04</t>
+  </si>
+  <si>
+    <t>Grow-shroom</t>
+  </si>
+  <si>
+    <t>05, 06</t>
   </si>
 </sst>
 </file>
@@ -898,7 +904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B48151-CA72-4105-BB43-B9D654C6E679}">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.21875" style="3" customWidth="1"/>
@@ -1194,6 +1200,17 @@
         <v>28</v>
       </c>
     </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M16">
     <sortCondition ref="A1:A16"/>

</xml_diff>

<commit_message>
Update - Wiki plant articles, Batch 8
Added art for Solar Flare and The Pinearch
</commit_message>
<xml_diff>
--- a/art/art_direction.xlsx
+++ b/art/art_direction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\art\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85AEE0C4-3B63-422A-8F25-93E9982FE4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310A0A19-5903-4157-9522-1B1EE26E9997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="86">
   <si>
     <t>Black</t>
   </si>
@@ -202,9 +202,6 @@
     <t>03, 05</t>
   </si>
   <si>
-    <t>Sun-shroom &amp; Sunnier-shroom</t>
-  </si>
-  <si>
     <t>Yellow 01 used for base, Yellow 02 used for pattern</t>
   </si>
   <si>
@@ -232,9 +229,6 @@
     <t>Grey 02 used for base, Grey 03 used for pattern</t>
   </si>
   <si>
-    <t>Pineclone</t>
-  </si>
-  <si>
     <t>Full Black</t>
   </si>
   <si>
@@ -278,6 +272,18 @@
   </si>
   <si>
     <t>05, 06</t>
+  </si>
+  <si>
+    <t>Solar Flare</t>
+  </si>
+  <si>
+    <t>02, 06</t>
+  </si>
+  <si>
+    <t>Pineclone, The Pinearch</t>
+  </si>
+  <si>
+    <t>Sun-shroom, Sunnier-shroom</t>
   </si>
 </sst>
 </file>
@@ -693,29 +699,29 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -750,7 +756,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>51</v>
@@ -791,7 +797,7 @@
     </row>
     <row r="12" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M12" s="4" t="s">
         <v>31</v>
@@ -799,7 +805,7 @@
     </row>
     <row r="13" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>30</v>
@@ -826,7 +832,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>51</v>
@@ -862,7 +868,7 @@
         <v>20</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
@@ -876,7 +882,7 @@
         <v>22</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
@@ -904,16 +910,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B48151-CA72-4105-BB43-B9D654C6E679}">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.21875" style="3" customWidth="1"/>
-    <col min="2" max="12" width="8.33203125" style="4" customWidth="1"/>
+    <col min="2" max="12" width="8.88671875" style="4" customWidth="1"/>
     <col min="13" max="13" width="72.21875" style="4" customWidth="1"/>
     <col min="14" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="2" customFormat="1" ht="16.2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" s="2" customFormat="1" ht="32.4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -974,7 +980,7 @@
         <v>14</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -1024,7 +1030,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>13</v>
@@ -1045,175 +1051,198 @@
         <v>13</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>22</v>
+        <v>80</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>81</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="J7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K7" s="4" t="s">
+    </row>
+    <row r="8" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>33</v>
+      <c r="M8" s="4" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="F9" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="J10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K10" s="4" t="s">
+      <c r="J11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="4" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="M12" s="4" t="s">
+    </row>
+    <row r="13" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M13" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M14" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="4" t="s">
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>51</v>
+      <c r="G15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>79</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="M15" s="4" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>51</v>
       </c>
+      <c r="L17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M16">
-    <sortCondition ref="A1:A16"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M18">
+    <sortCondition ref="A1:A18"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>